<commit_message>
mise en forme de toute la partie adhésion
</commit_message>
<xml_diff>
--- a/Comparaison_Hebergeur_Web.xlsx
+++ b/Comparaison_Hebergeur_Web.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acout\Desktop\projet_etu\Stage_annee_2\Stage_annee_2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D6A1016-892D-44D2-B1B6-14397AE7E1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F561540-04A6-4CA6-BF77-EFE72ED2F67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{CAEC590B-3AD9-4176-AE10-DD277B79CFA1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CAEC590B-3AD9-4176-AE10-DD277B79CFA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -247,16 +247,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,7 +599,7 @@
   <sheetFormatPr defaultColWidth="25.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="9" width="25.109375" style="1"/>
-    <col min="10" max="10" width="25.109375" style="2"/>
+    <col min="10" max="10" width="25.109375" style="4"/>
     <col min="11" max="16384" width="25.109375" style="1"/>
   </cols>
   <sheetData>
@@ -625,7 +628,7 @@
       <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -657,16 +660,16 @@
       <c r="G2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="L2" s="1" t="s">
@@ -701,7 +704,7 @@
       <c r="I3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>45</v>
       </c>
       <c r="K3" s="1" t="s">
@@ -730,19 +733,19 @@
       <c r="F4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="2" t="s">
         <v>49</v>
       </c>
       <c r="L4" s="1" t="s">
@@ -777,10 +780,10 @@
       <c r="I5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="2" t="s">
         <v>50</v>
       </c>
       <c r="L5" s="1" t="s">

</xml_diff>